<commit_message>
Upgrade stock price simulation to Monte Carlo method
- 기존의 단순 평균/표준편차 덧셈 기반의 5일 가격 예측 모델을 폐기하고, numpy 정규분포 난수를 활용한 10,000회 몬테카를로 시뮬레이션(Monte Carlo Simulation) 알고리즘으로 전면 교체
- 통계적 신뢰도 확보를 위해 하위 10%(비관적), 중간값 50%(중립), 상위 10%(낙관적) 백분위수를 추출하여 UI에 표시하도록 개선
</commit_message>
<xml_diff>
--- a/home/src/Daily_Economic_Report_20260702.xlsx
+++ b/home/src/Daily_Economic_Report_20260702.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8019.22</v>
+        <v>7993.68</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.42</v>
+        <v>-3.73</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1554.48</v>
+        <v>1553.68</v>
       </c>
       <c r="C5" t="n">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -522,10 +522,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67.56</v>
+        <v>67.70999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.79</v>
+        <v>-2.58</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -625,15 +625,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>28,920원</t>
+          <t>28,930원</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -643,17 +643,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28,920원</t>
+          <t>28,930원</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28,297원</t>
+          <t>28,298원</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27,474원</t>
+          <t>27,483원</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -683,15 +683,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>205,925원</t>
+          <t>205,910원</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-0.89</v>
+        <v>-0.9</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>201,934원</t>
+          <t>201,933원</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -741,15 +741,15 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15,695원</t>
+          <t>15,702원</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>77%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -799,11 +799,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>33,160원</t>
+          <t>33,190원</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>32,860원</t>
+          <t>32,861원</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -857,15 +857,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>66,455원</t>
+          <t>66,425원</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>-3.75</v>
+        <v>-3.79</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>59%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>65,437원</t>
+          <t>65,435원</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -915,15 +915,15 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13,130원</t>
+          <t>13,090원</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>-0.11</v>
+        <v>-0.42</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>12,811원</t>
+          <t>12,809원</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -973,15 +973,15 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>298,000원</t>
+          <t>296,750원</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>-5.25</v>
+        <v>-5.64</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>329,250원</t>
+          <t>329,187원</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1031,15 +1031,15 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2,397,000원</t>
+          <t>2,387,000원</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-6.37</v>
+        <v>-6.76</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>59%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2,452,750원</t>
+          <t>2,452,250원</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1089,15 +1089,15 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>498,500원</t>
+          <t>494,500원</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2.26</v>
+        <v>1.44</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>62%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>573,275원</t>
+          <t>573,075원</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4700</v>
+        <v>3600</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>146,200원</t>
+          <t>145,100원</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3.32</v>
+        <v>2.54</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>152,290원</t>
+          <t>152,235원</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1263,11 +1263,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1,423,000원</t>
+          <t>1,417,000원</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1.93</v>
+        <v>1.5</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1,346,850원</t>
+          <t>1,346,550원</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1321,15 +1321,15 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>172,400원</t>
+          <t>171,800원</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8.77</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1339,17 +1339,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>172,400원</t>
+          <t>172,000원</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>158,945원</t>
+          <t>158,915원</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>163,780원</t>
+          <t>163,400원</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>77%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1843,15 +1843,15 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>359,500원</t>
+          <t>358,500원</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3.3</v>
+        <v>3.02</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>384,350원</t>
+          <t>384,300원</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1901,15 +1901,15 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>486,500원</t>
+          <t>486,000원</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>-0.92</v>
+        <v>-1.02</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>512,625원</t>
+          <t>512,600원</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1959,20 +1959,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>126,300원</t>
+          <t>125,800원</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>-4.82</v>
+        <v>-5.2</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>126,300원</t>
+          <t>125,800원</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>159,885원</t>
+          <t>159,860원</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2017,15 +2017,15 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>15,955원</t>
+          <t>15,970원</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>-0.22</v>
+        <v>-0.13</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>42%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2075,15 +2075,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>13,955원</t>
+          <t>13,965원</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-0.21</v>
+        <v>-0.14</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>146%</t>
+          <t>165%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2133,20 +2133,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>223,500원</t>
+          <t>222,500원</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-9.33</v>
+        <v>-9.74</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>223,500원</t>
+          <t>222,500원</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>284,250원</t>
+          <t>284,200원</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2219,7 +2219,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 20:52:00 GMT</t>
+          <t>Wed, 01 Jul 2026 20:51:58 GMT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2354,17 +2354,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 21:55:00 GMT</t>
+          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(출연) [스타트 경제] 환율, 또 금융위기 후 최고...장중 1,560원까지 위협</t>
+          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2374,24 +2374,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE15ZW9lYkUwVlpRN2lvTUlTUzFvSThLM0VtQkpHQVBvY3lqVDhFNkpnWE03LWtpT05od1NiN0lrRG9LdWJLZzZrcFl5VU00WEJyWS1kb3hmSUJMcF90Mnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
+          <t>Wed, 01 Jul 2026 21:55:00 GMT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
+          <t>(출연) [스타트 경제] 환율, 또 금융위기 후 최고...장중 1,560원까지 위협</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2401,61 +2401,61 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE15ZW9lYkUwVlpRN2lvTUlTUzFvSThLM0VtQkpHQVBvY3lqVDhFNkpnWE03LWtpT05od1NiN0lrRG9LdWJLZzZrcFl5VU00WEJyWS1kb3hmSUJMcF90Mnc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 02:07:08 GMT</t>
+          <t>Wed, 01 Jul 2026 23:21:23 GMT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KB Think</t>
+          <t>지디넷코리아</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>日 국채금리 일제히 상승…10년물 표면금리 29년 만에 최고</t>
+          <t>美 반도체 주식 무더기 폭락…"메타발 악재 직격탄"</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>긍정적 (호재)</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9IajBWQVpGaFlaLWhTWFJsMk16VERDa0twdmo1em5jNXFNejB0THNXWU5OM0p3cW9EVWN2ZmgxR0NxZWZjMXpUelltcG5hYWxyS2c0Z1YtNXBUVWtiMnJUT2RXMEhwMWxUNTBOcDlmTG1WZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9qWE54WjVNbDhCTmxtcW5FVllWTFBTSXdNZ2ZNczhNd3BtdjJ5dUNzZmpldHBDdGpHSWJOeDZzY2RhcndYNnZIRFFYZWhWY2tQLV9KX3hR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:21:23 GMT</t>
+          <t>Thu, 02 Jul 2026 02:07:08 GMT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>지디넷코리아</t>
+          <t>KB Think</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>美 반도체 주식 무더기 폭락…"메타발 악재 직격탄"</t>
+          <t>日 국채금리 일제히 상승…10년물 표면금리 29년 만에 최고</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9qWE54WjVNbDhCTmxtcW5FVllWTFBTSXdNZ2ZNczhNd3BtdjJ5dUNzZmpldHBDdGpHSWJOeDZzY2RhcndYNnZIRFFYZWhWY2tQLV9KX3hR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9IajBWQVpGaFlaLWhTWFJsMk16VERDa0twdmo1em5jNXFNejB0THNXWU5OM0p3cW9EVWN2ZmgxR0NxZWZjMXpUelltcG5hYWxyS2c0Z1YtNXBUVWtiMnJUT2RXMEhwMWxUNTBOcDlmTG1WZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2678,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:03:22 GMT</t>
+          <t>Thu, 02 Jul 2026 03:24:29 GMT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[변액보험 상반기] 주식시장 훈풍 지속…라이나생명 수익률 선두</t>
+          <t>핌코 "AI, 실질 중립금리 높이는 게 아니라 낮춘다…안전자산 수요↑"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2698,14 +2698,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFAxUmxPSzFMak9XZ2htaVhTeTR4OHpmaTNlMWZVOWdGSjJDdGpxZndXY3A1RHhobW9RSEpzNEN4emE3cktIVDdYNndPMGpRRl9xa2FuS1JOWEU3WGI4LVdtcWYzVk41RzY4aHJtVS10OUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5mbGc1dVh4WVd0NHlEOTlIV3luZFhlcGFBUVBDQ2tWeUozTURjaUNBSjhydUI2RDIyN2hiaFM1QllDM2JoaV9WZWxyTmhyWDFMQjZIbm4wc1BTY2U0VVVMRzEta3NNM1Q1UGt1NUh0b3M?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mon, 29 Jun 2026 01:39:00 GMT</t>
+          <t>Thu, 02 Jul 2026 00:03:22 GMT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>"한은 최종금리 3.5% 아닌 3.25%에 그칠 가능성…달러 조달여건도 양호"</t>
+          <t>[변액보험 상반기] 주식시장 훈풍 지속…라이나생명 수익률 선두</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2725,14 +2725,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE90NHFrMWthSmZqZG1XTXVLWHhCWG5EbEtGcHpkOXJ6UXl2NUlMQ18wdGJGTmdIc2tpN3VtMzRha09GUXNibkpIVDY3bjRmT3NrUlV1c3dXZXFQdXptX2NuNElkVEtNYVd0STg3b2JmOTM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFAxUmxPSzFMak9XZ2htaVhTeTR4OHpmaTNlMWZVOWdGSjJDdGpxZndXY3A1RHhobW9RSEpzNEN4emE3cktIVDdYNndPMGpRRl9xa2FuS1JOWEU3WGI4LVdtcWYzVk41RzY4aHJtVS10OUw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 01:29:10 GMT</t>
+          <t>Mon, 29 Jun 2026 01:39:00 GMT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>미래에셋, 국내주식 증거금률 40%로 상향…"쏠림 선제 대응"</t>
+          <t>"한은 최종금리 3.5% 아닌 3.25%에 그칠 가능성…달러 조달여건도 양호"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0tWlFWVmpna1NVMzJ1OEljNmlJSkMwdzBsbzBMZHlfRXp5VXAyTUhwVG44WWMtX2l4MGhZdU5vSnp5bTVpclR6VlN4UUc5UkxVTWZYVzQxZ0RiZmJibW5xM0ljOFJLREF2Y2ZsTkZoaV8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE90NHFrMWthSmZqZG1XTXVLWHhCWG5EbEtGcHpkOXJ6UXl2NUlMQ18wdGJGTmdIc2tpN3VtMzRha09GUXNibkpIVDY3bjRmT3NrUlV1c3dXZXFQdXptX2NuNElkVEtNYVd0STg3b2JmOTM?oc=5</t>
         </is>
       </c>
     </row>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AI, 반도체</t>
+          <t>🛍️소비/매출폭발, 반도체, AI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>✈️유가하락수혜, 🌱성수기/계절수혜, 환율</t>
+          <t>🌱성수기/계절수혜, ✈️유가하락수혜, 환율</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2890,11 +2890,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.63</v>
+        <v>3.14</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KB금융 (+8.77%)</t>
+          <t>KB금융 (+8.39%)</t>
         </is>
       </c>
     </row>
@@ -2905,41 +2905,41 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TIGER 미국S&amp;P500 (+0.19%)</t>
+          <t>TIGER 미국S&amp;P500 (+0.23%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>신흥국(알파)</t>
+          <t>헷징/안전자산</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.11</v>
+        <v>-0.14</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TIGER 인도니프티50 (-0.11%)</t>
+          <t>KODEX 미국달러선물 (-0.13%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>헷징/안전자산</t>
+          <t>신흥국(알파)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.22</v>
+        <v>-0.42</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TIGER 미국채10년선물 (-0.21%)</t>
+          <t>TIGER 인도니프티50 (-0.42%)</t>
         </is>
       </c>
     </row>
@@ -2950,11 +2950,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.02</v>
+        <v>-1.13</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LG에너지솔루션 (+3.3%)</t>
+          <t>LG에너지솔루션 (+3.02%)</t>
         </is>
       </c>
     </row>
@@ -2965,11 +2965,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.29</v>
+        <v>-2.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>삼성바이오로직스 (+1.93%)</t>
+          <t>NAVER (+1.57%)</t>
         </is>
       </c>
     </row>
@@ -2995,11 +2995,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-5.25</v>
+        <v>-5.64</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>삼성전자 (-5.25%)</t>
+          <t>삼성전자 (-5.64%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add average purchase price tracking and UI/Telegram updates
- 사용자가 종목을 추가할 때 '매수 단가(평단가)'를 입력받아 custom_portfolio.json에 저장하는 로직 추가
- GUI의 '나의 실제 보유 주식 현황' 목록(tv_my)에 [매수 단가], [수익률(%)] 컬럼을 신설하여 직관적 파악 가능
- 텔레그램 알림 전송(send_briefing_to_telegram) 시 종목별 현재가, 매수 단가, 수익률(%) 포맷을 적용하여 보고서 가독성 강화
</commit_message>
<xml_diff>
--- a/home/src/Daily_Economic_Report_20260702.xlsx
+++ b/home/src/Daily_Economic_Report_20260702.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7993.68</v>
+        <v>7955.91</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.73</v>
+        <v>-4.19</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1553.68</v>
+        <v>1551.48</v>
       </c>
       <c r="C5" t="n">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -522,10 +522,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67.70999999999999</v>
+        <v>68.58</v>
       </c>
       <c r="C6" t="n">
-        <v>-2.58</v>
+        <v>-1.32</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,50 +560,55 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>매수 단가</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>일간 변동금액</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>현재가(원/$)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>전일비(%)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>거래량 증감(%)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>예상 저점(지지선)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>예상 고점(저항선)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>목표 매수가</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>부분 매도가</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>투자 성향</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>AI 매매 시그널</t>
         </is>
@@ -623,45 +628,48 @@
       <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>28,930원</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>55%</t>
-        </is>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>28,935원</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.24</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>27,695원</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>28,930원</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>28,935원</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>28,298원</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>27,483원</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>27,488원</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>코어(필수)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -679,47 +687,50 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>-0</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>205,910원</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>-0.9</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>63%</t>
-        </is>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>205,790원</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.96</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>69%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>194,530원</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>207,780원</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>201,933원</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>201,927원</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>197,391원</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -739,45 +750,48 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>15,702원</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>78%</t>
-        </is>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>15,690원</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.13</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>81%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>15,360원</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15,834원</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>15,589원</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>15,042원</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>배당/가치(안전)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -797,45 +811,48 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>33,190원</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>58%</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>31,070원</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>34,860원</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>32,861원</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>33,117원</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -853,47 +870,50 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
         <v>-0</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>66,425원</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>-3.79</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>66,270원</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>-4.02</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>60,190원</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>69,480원</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>65,435원</t>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>65,427원</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>66,006원</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -911,47 +931,50 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
         <v>-0</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>13,090원</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>45%</t>
-        </is>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>13,120원</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.19</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>12,175원</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>13,185원</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>12,809원</t>
-        </is>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>12,810원</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>12,525원</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>신흥국(알파)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>⚠️ 단기 고점 (매도 준비/관망)</t>
         </is>
@@ -969,47 +992,50 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
         <v>-0</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>296,750원</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>-5.64</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>66%</t>
-        </is>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>295,500원</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>-6.04</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>69%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>295,500원</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>362,500원</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>329,187원</t>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>329,125원</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>344,375원</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>국내 우량주</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1027,47 +1053,50 @@
         </is>
       </c>
       <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
         <v>-0</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2,387,000원</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>-6.76</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>59%</t>
-        </is>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2,368,000원</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>-7.5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>1,911,000원</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>2,919,000원</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2,452,250원</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>2,451,300원</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>2,773,050원</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1087,45 +1116,48 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>494,500원</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>62%</t>
-        </is>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>494,000원</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1.33</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>480,500원</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>700,000원</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>573,075원</t>
-        </is>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t>573,050원</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>665,000원</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>배당/가치(안전)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1143,47 +1175,50 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3600</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>145,100원</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>52%</t>
-        </is>
+        <v>168300</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>146,000원</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>3.18</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>135,300원</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>170,200원</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>152,235원</t>
-        </is>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t>152,280원</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>161,690원</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>배당/가치(안전)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1203,45 +1238,48 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>200,500원</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>26%</t>
-        </is>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>201,500원</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2.08</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>196,400원</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>279,000원</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>225,420원</t>
-        </is>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
+          <t>225,470원</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>265,050원</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1261,45 +1299,48 @@
       <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1,417,000원</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>53%</t>
-        </is>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1,420,000원</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1.72</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>1,243,000원</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>1,448,000원</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>1,346,550원</t>
-        </is>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>1,346,700원</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>1,375,600원</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -1319,45 +1360,48 @@
       <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>171,800원</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>8.390000000000001</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>90%</t>
-        </is>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>171,500원</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>149,300원</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>172,000원</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>158,915원</t>
-        </is>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t>158,900원</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
           <t>163,400원</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>배당/가치(안전)</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -1375,47 +1419,50 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
         <v>-0</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>$68.88</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>-0.29</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>48%</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>$65.65</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>$69.30</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>$67.30</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>$65.84</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>기후/식량(방어)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -1433,47 +1480,50 @@
         </is>
       </c>
       <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
         <v>-0</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>$78.99</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>-0.27</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>41%</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>$76.54</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>$80.24</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>$78.25</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>$76.23</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>기후/식량(방어)</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -1491,47 +1541,50 @@
         </is>
       </c>
       <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
         <v>-0</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>7,260원</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>-1.63</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>6,920원</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>8,280원</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>7,532원</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>7,866원</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>기후/식량(방어)</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1549,47 +1602,50 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-4400</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>5,090원</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>-7.96</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>77%</t>
-        </is>
+        <v>5060</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-4600</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5,070원</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>-8.32</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>78%</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>4,155원</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>6,030원</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>4,710원</t>
-        </is>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t>4,709원</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>5,728원</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>기후/식량(방어)</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>✅ 보유 및 분할 매수</t>
         </is>
@@ -1607,47 +1663,50 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
         <v>-0</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>$43.18</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>-1.19</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>79%</t>
-        </is>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>$42.35</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>$50.39</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>$45.75</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>$47.87</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1665,47 +1724,50 @@
         </is>
       </c>
       <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
         <v>-0</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>$87.66</t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>-0.95</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>44%</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>$85.13</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>$98.32</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>$91.81</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>$93.40</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1723,47 +1785,50 @@
         </is>
       </c>
       <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
         <v>-0</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>$77.97</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>-0.4</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>62%</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>$75.60</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>$84.50</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>$79.83</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>$80.27</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1781,47 +1846,50 @@
         </is>
       </c>
       <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
         <v>-0</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>$75.29</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>-2.18</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>70%</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>120%</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>$75.29</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>$89.94</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>$81.85</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>$85.45</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1841,45 +1909,48 @@
       <c r="C23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>358,500원</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>47%</t>
-        </is>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>357,000원</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2.59</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>331,500원</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>420,500원</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>384,300원</t>
-        </is>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
+          <t>384,225원</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
           <t>399,475원</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1897,47 +1968,50 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
         <v>-0</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>486,000원</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>-1.02</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>51%</t>
-        </is>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>485,000원</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>-1.22</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>53%</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>455,000원</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>568,000원</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>512,600원</t>
-        </is>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
+          <t>512,550원</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>539,600원</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -1955,47 +2029,50 @@
         </is>
       </c>
       <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
         <v>-0</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>125,800원</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>56%</t>
-        </is>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>125,400원</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>-5.5</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>125,800원</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
+          <t>125,400원</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>186,500원</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>159,860원</t>
-        </is>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>159,840원</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>177,175원</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>미래자원/배터리</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -2013,47 +2090,50 @@
         </is>
       </c>
       <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
         <v>-0</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>15,970원</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>-0.13</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>42%</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>15,505원</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>15,990원</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>15,729원</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>15,190원</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>헷징/안전자산</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>⚠️ 단기 고점 (매도 준비/관망)</t>
         </is>
@@ -2071,47 +2151,50 @@
         </is>
       </c>
       <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
         <v>-0</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>13,965원</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>-0.14</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>165%</t>
-        </is>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>13,960원</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>-0.18</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>179%</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>13,535원</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>14,005원</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>13,775원</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>13,304원</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>헷징/안전자산</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>⚠️ 단기 고점 (매도 준비/관망)</t>
         </is>
@@ -2129,47 +2212,50 @@
         </is>
       </c>
       <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
         <v>-0</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>222,500원</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>56%</t>
-        </is>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>222,000원</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>-9.94</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>222,500원</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
+          <t>222,000원</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>361,000원</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>284,200원</t>
-        </is>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
+          <t>284,175원</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
           <t>342,950원</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -2273,71 +2359,71 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 22:13:11 GMT</t>
+          <t>Thu, 02 Jul 2026 01:47:58 GMT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[증시전략] 메모리 가격 하락?…삼전닉스 팔까 말까, 전망은?</t>
+          <t>"우대금리와 함께 쿠폰도 챙기세요"…iM뱅크, '착착통장' 출시</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBZeklJWEthcGdoNF92TmtyWVJDYVV6QWpNS1YzajM1eVBQVlhYdUZFYjF5RG9JbkN4MkpBT3pBR1pUd3Z4ZVBIamxYbHo2VlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBudm5PQjE0R19pVnBxVHl3OWxGbnF0YnlhMzVJRFBDNm5PNFNzTlQ1aldtczRDTDMzdkFpZWMya3M4OG9SSFlyWi1rTHZwU0c2WkE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 01:47:58 GMT</t>
+          <t>Wed, 01 Jul 2026 22:13:11 GMT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>v.daum.net</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>"우대금리와 함께 쿠폰도 챙기세요"…iM뱅크, '착착통장' 출시</t>
+          <t>[증시전략] 메모리 가격 하락?…삼전닉스 팔까 말까, 전망은?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBudm5PQjE0R19pVnBxVHl3OWxGbnF0YnlhMzVJRFBDNm5PNFNzTlQ1aldtczRDTDMzdkFpZWMya3M4OG9SSFlyWi1rTHZwU0c2WkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBZeklJWEthcGdoNF92TmtyWVJDYVV6QWpNS1YzajM1eVBQVlhYdUZFYjF5RG9JbkN4MkpBT3pBR1pUd3Z4ZVBIamxYbHo2VlE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:13:35 GMT</t>
+          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>한성숙, 첫 비상경제점검회의 주재‥"호르무즈 남은 2척 끝까지 챙길 것"</t>
+          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2347,24 +2433,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE83eVk4a0VLNTI3VzAxcTlycUxMaktwTElrTE51UThSU0lhZk5BeGJwM0lpY1NmNGFwUWJ1MDBnQVEtbjVIYVRYeW16dzljckhiQ2laMTlVUlVGVjh3Z1Q1Z1FVb3I0Q0hRanh5NkhLcGZJQ2lMbWJOZ9IBeEFVX3lxTE1FNDJ4Ymk0MWR3UlVYcC0xTXNCbnVMUUxmeXY3NXVwZVRuMnE3a2tNZ0xsVVZZZVNkRUJqWG1yRG1Xc1dWa1o1U0MxX1JUMWd4ODJ1R01NeTBZd0RiRllVbndPdHNEVXEzQjVYcmo3TlhtT0RRV3RZcg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
+          <t>Thu, 02 Jul 2026 00:13:35 GMT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
+          <t>한성숙, 첫 비상경제점검회의 주재‥"호르무즈 남은 2척 끝까지 챙길 것"</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2374,7 +2460,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE83eVk4a0VLNTI3VzAxcTlycUxMaktwTElrTE51UThSU0lhZk5BeGJwM0lpY1NmNGFwUWJ1MDBnQVEtbjVIYVRYeW16dzljckhiQ2laMTlVUlVGVjh3Z1Q1Z1FVb3I0Q0hRanh5NkhLcGZJQ2lMbWJOZ9IBeEFVX3lxTE1FNDJ4Ymk0MWR3UlVYcC0xTXNCbnVMUUxmeXY3NXVwZVRuMnE3a2tNZ0xsVVZZZVNkRUJqWG1yRG1Xc1dWa1o1U0MxX1JUMWd4ODJ1R01NeTBZd0RiRllVbndPdHNEVXEzQjVYcmo3TlhtT0RRV3RZcg?oc=5</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2602,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:41:39 GMT</t>
+          <t>Wed, 01 Jul 2026 23:06:08 GMT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>오늘의 증시</t>
+          <t>워시 "생애 최대 경제 격변기…AI 혁명 1∼2회"</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2536,78 +2622,78 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFA1MWtmcmxtYUU4NGlyQTdmbG5uLWhtbXpwMTNqZU4yOE0zX1g3Z0lKc1I5VnJvYjgzeFZ2WG9sWU9ZNDhtR0xPSlNaWTN1Vk9reEhhbXJGSWhaOFY1Y3ZsSEs2UUxmVlRMNUUwQTdlaDk3OHg3QXp3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE4taGJydHRfVmgwU0puMDI4T243UlE5WjZqcTlLTXp1bkNXNS1NbmN0a2tEQ3otU0xqRFdPMWZhR0pQc1NqcEFzQWN6SWhiUHJuWG53cWQ1TzVTaFnSAWBBVV95cUxOTDNqODVBaHRyUi1SRnQ4SWh2TXJwZ1RtNXRzbzJJbS1iUTRMNDA1ZUJvNlF0aVlpTlFwaTdwNndSZFROSEJIcHZNNm96ZF9WZl8wLTFxLWNLOU53bUMtNzE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:06:08 GMT</t>
+          <t>Wed, 01 Jul 2026 20:58:01 GMT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>v.daum.net</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>워시 "생애 최대 경제 격변기…AI 혁명 1∼2회"</t>
+          <t>[뉴욕증시]반도체 업종 울자 일제히 하락 마감…워시 발언에 주목</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE4taGJydHRfVmgwU0puMDI4T243UlE5WjZqcTlLTXp1bkNXNS1NbmN0a2tEQ3otU0xqRFdPMWZhR0pQc1NqcEFzQWN6SWhiUHJuWG53cWQ1TzVTaFnSAWBBVV95cUxOTDNqODVBaHRyUi1SRnQ4SWh2TXJwZ1RtNXRzbzJJbS1iUTRMNDA1ZUJvNlF0aVlpTlFwaTdwNndSZFROSEJIcHZNNm96ZF9WZl8wLTFxLWNLOU53bUMtNzE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBBdmYzcUE2TEtFMmpIRlc5X0VndUljeWZUa0Q5MXJWemU2YVk4ekJzM29jclotY1VBb21kdXlUbmczUDZwcWNNYnRiLWYwQW8?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 20:58:01 GMT</t>
+          <t>Thu, 02 Jul 2026 00:44:51 GMT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[뉴욕증시]반도체 업종 울자 일제히 하락 마감…워시 발언에 주목</t>
+          <t>어린이 경제박사 되세요... 11일 경제교실 개최</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBBdmYzcUE2TEtFMmpIRlc5X0VndUljeWZUa0Q5MXJWemU2YVk4ekJzM29jclotY1VBb21kdXlUbmczUDZwcWNNYnRiLWYwQW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9XblNZWWkxaUNIcVZDaEpEbldHbWJwa29mSXhtck9ac3NYUm0tR1VKQlhxOWRHRElmcEpjUThWVlpGLUtvNFRKRDA1NXdnaG1RV0E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:44:51 GMT</t>
+          <t>Thu, 02 Jul 2026 03:24:15 GMT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>어린이 경제박사 되세요... 11일 경제교실 개최</t>
+          <t>오늘의 증시</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2617,7 +2703,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9XblNZWWkxaUNIcVZDaEpEbldHbWJwa29mSXhtck9ac3NYUm0tR1VKQlhxOWRHRElmcEpjUThWVlpGLUtvNFRKRDA1NXdnaG1RV0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE9zY29PWF95SVJpSXQyN3owdFh4V1hFbWtqVGEtYkpmY0pEbjZRWDMyRzc2S2txWHNMQ1ItZDFrRTEtYkFieDlsejFWSXlMSkt4TWthZ1JGazgzSVFVTTFrV2lLVUdKdmE1TUxFMGY5U1ZTMFJYcDBRag?oc=5</t>
         </is>
       </c>
     </row>
@@ -2800,7 +2886,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>🛍️소비/매출폭발, 반도체, AI</t>
+          <t>AI, 반도체, 🛍️소비/매출폭발</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2820,7 +2906,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>🌱성수기/계절수혜, ✈️유가하락수혜, 환율</t>
+          <t>✈️유가하락수혜, 환율, 🌱성수기/계절수혜</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2890,11 +2976,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.14</v>
+        <v>3.21</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KB금융 (+8.39%)</t>
+          <t>KB금융 (+8.2%)</t>
         </is>
       </c>
     </row>
@@ -2905,11 +2991,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TIGER 미국S&amp;P500 (+0.23%)</t>
+          <t>TIGER 미국S&amp;P500 (+0.24%)</t>
         </is>
       </c>
     </row>
@@ -2920,7 +3006,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.14</v>
+        <v>-0.16</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2935,11 +3021,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.42</v>
+        <v>-0.19</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TIGER 인도니프티50 (-0.42%)</t>
+          <t>TIGER 인도니프티50 (-0.19%)</t>
         </is>
       </c>
     </row>
@@ -2950,11 +3036,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.13</v>
+        <v>-1.26</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LG에너지솔루션 (+3.02%)</t>
+          <t>LG에너지솔루션 (+2.59%)</t>
         </is>
       </c>
     </row>
@@ -2965,11 +3051,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.46</v>
+        <v>-2.53</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NAVER (+1.57%)</t>
+          <t>NAVER (+2.08%)</t>
         </is>
       </c>
     </row>
@@ -2980,7 +3066,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2.54</v>
+        <v>-2.63</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2995,11 +3081,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-5.64</v>
+        <v>-6.04</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>삼성전자 (-5.64%)</t>
+          <t>삼성전자 (-6.04%)</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3143,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5,090원</t>
+          <t>5,070원</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3066,7 +3152,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>12.5</v>
+        <v>13</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add daily detailed breakdown to Telegram simulation report
- 텔레그램 알림 메시지에서 향후 5일 주가 시뮬레이션 전송 시, 마지막 5일차 결과만 출력되던 버그 수정
- UI(앱)에서와 동일하게 향후 1일차부터 5일차까지 매일매일의 시나리오(하락/중립/상승)를 일자별(MM/DD)로 구분하여 전송하도록 포맷 변경
</commit_message>
<xml_diff>
--- a/home/src/Daily_Economic_Report_20260702.xlsx
+++ b/home/src/Daily_Economic_Report_20260702.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7955.91</v>
+        <v>7947.15</v>
       </c>
       <c r="C2" t="n">
-        <v>-4.19</v>
+        <v>-4.29</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1551.48</v>
+        <v>1550.88</v>
       </c>
       <c r="C5" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -522,14 +522,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68.58</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>-1.32</v>
+        <v>-1.22</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
     </row>
@@ -633,15 +633,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,935원</t>
+          <t>28,910원</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -651,17 +651,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28,935원</t>
+          <t>28,910원</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28,298원</t>
+          <t>28,297원</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>27,488원</t>
+          <t>27,464원</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -694,15 +694,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>205,790원</t>
+          <t>205,755원</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>-0.96</v>
+        <v>-0.97</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>71%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>201,927원</t>
+          <t>201,925원</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -755,15 +755,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15,690원</t>
+          <t>15,685원</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15,589원</t>
+          <t>15,588원</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -816,11 +816,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>33,190원</t>
+          <t>33,165원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>32,861원</t>
+          <t>32,860원</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -877,15 +877,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>66,270원</t>
+          <t>66,205원</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-4.02</v>
+        <v>-4.11</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>65,427원</t>
+          <t>65,424원</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -938,15 +938,15 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13,120원</t>
+          <t>13,140원</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.19</v>
+        <v>-0.04</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>12,810원</t>
+          <t>12,811원</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -999,20 +999,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>295,500원</t>
+          <t>295,000원</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-6.04</v>
+        <v>-6.2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>71%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>295,500원</t>
+          <t>295,000원</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>329,125원</t>
+          <t>329,100원</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1060,15 +1060,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2,368,000원</t>
+          <t>2,364,000원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>-7.5</v>
+        <v>-7.66</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2,451,300원</t>
+          <t>2,451,100원</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1121,15 +1121,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>494,000원</t>
+          <t>493,000원</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1.33</v>
+        <v>1.13</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>573,050원</t>
+          <t>573,000원</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1178,19 +1178,19 @@
         <v>168300</v>
       </c>
       <c r="D11" t="n">
-        <v>4500</v>
+        <v>4900</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>146,000원</t>
+          <t>146,400원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3.18</v>
+        <v>3.46</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>152,280원</t>
+          <t>152,300원</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1304,15 +1304,15 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1,420,000원</t>
+          <t>1,419,000원</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.72</v>
+        <v>1.65</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,346,700원</t>
+          <t>1,346,650원</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>171,500원</t>
+          <t>171,200원</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>8.199999999999999</v>
+        <v>8.01</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>158,900원</t>
+          <t>158,885원</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1548,15 +1548,15 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>7,260원</t>
+          <t>7,250원</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-1.63</v>
+        <v>-1.76</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1605,19 +1605,19 @@
         <v>5060</v>
       </c>
       <c r="D18" t="n">
-        <v>-4600</v>
+        <v>-4700</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5,070원</t>
+          <t>5,060원</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-8.32</v>
+        <v>-8.5</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>4,709원</t>
+          <t>4,708원</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1975,15 +1975,15 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>485,000원</t>
+          <t>484,000원</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-1.22</v>
+        <v>-1.43</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>54%</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>512,550원</t>
+          <t>512,500원</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2036,11 +2036,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>125,400원</t>
+          <t>125,800원</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-5.5</v>
+        <v>-5.2</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>125,400원</t>
+          <t>125,800원</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>159,840원</t>
+          <t>159,860원</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2097,11 +2097,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15,970원</t>
+          <t>15,955원</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>-0.13</v>
+        <v>-0.22</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2158,15 +2158,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>13,960원</t>
+          <t>13,945원</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.18</v>
+        <v>-0.29</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>179%</t>
+          <t>181%</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>13,775원</t>
+          <t>13,774원</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2413,17 +2413,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
+          <t>Thu, 02 Jul 2026 00:13:35 GMT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
+          <t>한성숙, 첫 비상경제점검회의 주재‥"호르무즈 남은 2척 끝까지 챙길 것"</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2433,24 +2433,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE83eVk4a0VLNTI3VzAxcTlycUxMaktwTElrTE51UThSU0lhZk5BeGJwM0lpY1NmNGFwUWJ1MDBnQVEtbjVIYVRYeW16dzljckhiQ2laMTlVUlVGVjh3Z1Q1Z1FVb3I0Q0hRanh5NkhLcGZJQ2lMbWJOZ9IBeEFVX3lxTE1FNDJ4Ymk0MWR3UlVYcC0xTXNCbnVMUUxmeXY3NXVwZVRuMnE3a2tNZ0xsVVZZZVNkRUJqWG1yRG1Xc1dWa1o1U0MxX1JUMWd4ODJ1R01NeTBZd0RiRllVbndPdHNEVXEzQjVYcmo3TlhtT0RRV3RZcg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:13:35 GMT</t>
+          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>한성숙, 첫 비상경제점검회의 주재‥"호르무즈 남은 2척 끝까지 챙길 것"</t>
+          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE83eVk4a0VLNTI3VzAxcTlycUxMaktwTElrTE51UThSU0lhZk5BeGJwM0lpY1NmNGFwUWJ1MDBnQVEtbjVIYVRYeW16dzljckhiQ2laMTlVUlVGVjh3Z1Q1Z1FVb3I0Q0hRanh5NkhLcGZJQ2lMbWJOZ9IBeEFVX3lxTE1FNDJ4Ymk0MWR3UlVYcC0xTXNCbnVMUUxmeXY3NXVwZVRuMnE3a2tNZ0xsVVZZZVNkRUJqWG1yRG1Xc1dWa1o1U0MxX1JUMWd4ODJ1R01NeTBZd0RiRllVbndPdHNEVXEzQjVYcmo3TlhtT0RRV3RZcg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
         </is>
       </c>
     </row>
@@ -2602,17 +2602,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:06:08 GMT</t>
+          <t>Thu, 02 Jul 2026 00:41:39 GMT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>워시 "생애 최대 경제 격변기…AI 혁명 1∼2회"</t>
+          <t>오늘의 증시</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE4taGJydHRfVmgwU0puMDI4T243UlE5WjZqcTlLTXp1bkNXNS1NbmN0a2tEQ3otU0xqRFdPMWZhR0pQc1NqcEFzQWN6SWhiUHJuWG53cWQ1TzVTaFnSAWBBVV95cUxOTDNqODVBaHRyUi1SRnQ4SWh2TXJwZ1RtNXRzbzJJbS1iUTRMNDA1ZUJvNlF0aVlpTlFwaTdwNndSZFROSEJIcHZNNm96ZF9WZl8wLTFxLWNLOU53bUMtNzE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFA1MWtmcmxtYUU4NGlyQTdmbG5uLWhtbXpwMTNqZU4yOE0zX1g3Z0lKc1I5VnJvYjgzeFZ2WG9sWU9ZNDhtR0xPSlNaWTN1Vk9reEhhbXJGSWhaOFY1Y3ZsSEs2UUxmVlRMNUUwQTdlaDk3OHg3QXp3?oc=5</t>
         </is>
       </c>
     </row>
@@ -2656,17 +2656,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:44:51 GMT</t>
+          <t>Wed, 01 Jul 2026 23:06:08 GMT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>어린이 경제박사 되세요... 11일 경제교실 개최</t>
+          <t>워시 "생애 최대 경제 격변기…AI 혁명 1∼2회"</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2676,24 +2676,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9XblNZWWkxaUNIcVZDaEpEbldHbWJwa29mSXhtck9ac3NYUm0tR1VKQlhxOWRHRElmcEpjUThWVlpGLUtvNFRKRDA1NXdnaG1RV0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE4taGJydHRfVmgwU0puMDI4T243UlE5WjZqcTlLTXp1bkNXNS1NbmN0a2tEQ3otU0xqRFdPMWZhR0pQc1NqcEFzQWN6SWhiUHJuWG53cWQ1TzVTaFnSAWBBVV95cUxOTDNqODVBaHRyUi1SRnQ4SWh2TXJwZ1RtNXRzbzJJbS1iUTRMNDA1ZUJvNlF0aVlpTlFwaTdwNndSZFROSEJIcHZNNm96ZF9WZl8wLTFxLWNLOU53bUMtNzE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:24:15 GMT</t>
+          <t>Thu, 02 Jul 2026 00:44:51 GMT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>오늘의 증시</t>
+          <t>어린이 경제박사 되세요... 11일 경제교실 개최</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE9zY29PWF95SVJpSXQyN3owdFh4V1hFbWtqVGEtYkpmY0pEbjZRWDMyRzc2S2txWHNMQ1ItZDFrRTEtYkFieDlsejFWSXlMSkt4TWthZ1JGazgzSVFVTTFrV2lLVUdKdmE1TUxFMGY5U1ZTMFJYcDBRag?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9XblNZWWkxaUNIcVZDaEpEbldHbWJwa29mSXhtck9ac3NYUm0tR1VKQlhxOWRHRElmcEpjUThWVlpGLUtvNFRKRDA1NXdnaG1RV0E?oc=5</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AI, 반도체, 🛍️소비/매출폭발</t>
+          <t>AI, 🛍️소비/매출폭발, 반도체</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>✈️유가하락수혜, 환율, 🌱성수기/계절수혜</t>
+          <t>환율, 🌱성수기/계절수혜, ✈️유가하락수혜</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2976,11 +2976,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.21</v>
+        <v>3.18</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KB금융 (+8.2%)</t>
+          <t>KB금융 (+8.01%)</t>
         </is>
       </c>
     </row>
@@ -2991,41 +2991,41 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TIGER 미국S&amp;P500 (+0.24%)</t>
+          <t>TIGER 미국S&amp;P500 (+0.16%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>헷징/안전자산</t>
+          <t>신흥국(알파)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.16</v>
+        <v>-0.04</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KODEX 미국달러선물 (-0.13%)</t>
+          <t>TIGER 인도니프티50 (-0.04%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>신흥국(알파)</t>
+          <t>헷징/안전자산</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.19</v>
+        <v>-0.26</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TIGER 인도니프티50 (-0.19%)</t>
+          <t>KODEX 미국달러선물 (-0.22%)</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.26</v>
+        <v>-1.25</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.53</v>
+        <v>-2.59</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2.63</v>
+        <v>-2.7</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -3081,11 +3081,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-6.04</v>
+        <v>-6.2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>삼성전자 (-6.04%)</t>
+          <t>삼성전자 (-6.2%)</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5,070원</t>
+          <t>5,060원</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3152,7 +3152,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add domestic dividend stocks and Naver real-time scraping
- 기본 분석 포트폴리오에 국내 대표 고배당주(맥쿼리인프라, 기업은행, KT&G, SK텔레콤) 추가
- 야후 파이낸스의 한국 주식 가격 지연 문제 해결을 위해 네이버 증권 100% 실시간 크롤링 로직 도입
- 네이버 스크래핑 시 사용자의 환경 내 bs4(BeautifulSoup) 의존성 문제 및 타임아웃 지연 현상을 방지하기 위해 정규식(re) 방식으로 파서 교체
</commit_message>
<xml_diff>
--- a/home/src/Daily_Economic_Report_20260702.xlsx
+++ b/home/src/Daily_Economic_Report_20260702.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7947.15</v>
+        <v>7648.09</v>
       </c>
       <c r="C2" t="n">
-        <v>-4.29</v>
+        <v>-7.89</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1550.88</v>
+        <v>1548.28</v>
       </c>
       <c r="C5" t="n">
-        <v>0.15</v>
+        <v>-0.02</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -522,10 +522,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67.73999999999999</v>
+        <v>67.87</v>
       </c>
       <c r="C6" t="n">
-        <v>-1.22</v>
+        <v>-1.04</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,15 +633,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,910원</t>
+          <t>28,875원</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.16</v>
+        <v>0.03</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>63%</t>
+          <t>203%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -651,17 +651,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>28,910원</t>
+          <t>28,875원</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28,297원</t>
+          <t>28,295원</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>27,464원</t>
+          <t>27,431원</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>✅ 보유 및 분할 매수</t>
+          <t>🚀 거래량 급증 (수급 폭발)</t>
         </is>
       </c>
     </row>
@@ -694,15 +694,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>205,755원</t>
+          <t>204,595원</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>-0.97</v>
+        <v>-1.53</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>120%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>201,925원</t>
+          <t>201,867원</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -755,15 +755,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15,685원</t>
+          <t>15,725원</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>122%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15,588원</t>
+          <t>15,590원</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -816,15 +816,15 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>33,165원</t>
+          <t>33,050원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.82</v>
+        <v>0.47</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>106%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>32,860원</t>
+          <t>32,854원</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -877,15 +877,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>66,205원</t>
+          <t>65,270원</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-4.11</v>
+        <v>-5.47</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>66%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>65,424원</t>
+          <t>65,377원</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>✅ 보유 및 분할 매수</t>
+          <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
       </c>
     </row>
@@ -938,15 +938,15 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13,140원</t>
+          <t>13,130원</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.04</v>
+        <v>-0.11</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -999,20 +999,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>295,000원</t>
+          <t>286,000원</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-6.2</v>
+        <v>-9.06</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>135%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>295,000원</t>
+          <t>286,000원</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>329,100원</t>
+          <t>328,650원</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1060,15 +1060,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2,364,000원</t>
+          <t>2,187,000원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>-7.66</v>
+        <v>-14.57</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>137%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2,451,100원</t>
+          <t>2,442,250원</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1117,19 +1117,19 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>493,000원</t>
+          <t>482,000원</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1.13</v>
+        <v>-1.13</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>66%</t>
+          <t>104%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>573,000원</t>
+          <t>572,450원</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1178,19 +1178,19 @@
         <v>168300</v>
       </c>
       <c r="D11" t="n">
-        <v>4900</v>
+        <v>3700</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>146,400원</t>
+          <t>145,200원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3.46</v>
+        <v>2.61</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>122%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>152,300원</t>
+          <t>152,240원</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1243,15 +1243,15 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>201,500원</t>
+          <t>199,900원</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2.08</v>
+        <v>1.27</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>225,470원</t>
+          <t>225,390원</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1304,15 +1304,15 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1,419,000원</t>
+          <t>1,406,000원</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.65</v>
+        <v>0.72</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>105%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,346,650원</t>
+          <t>1,346,000원</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>171,200원</t>
+          <t>165,000원</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>8.01</v>
+        <v>4.1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>160%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>158,885원</t>
+          <t>158,575원</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1548,15 +1548,15 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>7,250원</t>
+          <t>7,160원</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-1.76</v>
+        <v>-2.98</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>65%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>7,532원</t>
+          <t>7,527원</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1605,19 +1605,19 @@
         <v>5060</v>
       </c>
       <c r="D18" t="n">
-        <v>-4700</v>
+        <v>-6300</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5,060원</t>
+          <t>4,900원</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-8.5</v>
+        <v>-11.39</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>118%</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>4,708원</t>
+          <t>4,700원</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1914,15 +1914,15 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>357,000원</t>
+          <t>354,000원</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.59</v>
+        <v>1.72</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>49%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>384,225원</t>
+          <t>384,075원</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1975,15 +1975,15 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>484,000원</t>
+          <t>470,500원</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-1.43</v>
+        <v>-4.18</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>512,500원</t>
+          <t>511,825원</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2036,20 +2036,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>125,800원</t>
+          <t>125,500원</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-5.2</v>
+        <v>-5.43</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>125,800원</t>
+          <t>125,500원</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>159,860원</t>
+          <t>159,845원</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2097,15 +2097,15 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15,955원</t>
+          <t>15,975원</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>-0.22</v>
+        <v>-0.09</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>15,729원</t>
+          <t>15,730원</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2158,15 +2158,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>13,945원</t>
+          <t>13,960원</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.29</v>
+        <v>-0.18</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>181%</t>
+          <t>252%</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>13,774원</t>
+          <t>13,775원</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2203,7 +2203,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>한미반도체 (사용자 추가)</t>
+          <t>맥쿼리인프라 (국내 인프라/고배당)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2219,43 +2219,287 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>222,000원</t>
+          <t>9,940원</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-9.94</v>
+        <v>-0.9</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>114%</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>222,000원</t>
+          <t>9,940원</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>10,704원</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>10,401원</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>10,168원</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>배당/가치(안전)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>✂️ 부분 매도 (고점대비 5%하락)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>기업은행 (국내 국책은행/고배당)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>20,600원</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>19,660원</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>23,100원</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>20,890원</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>21,945원</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>배당/가치(안전)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>✂️ 부분 매도 (고점대비 5%하락)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>KT&amp;G (국내 담배/경기방어/고배당)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>173,000원</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>167,100원</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>188,500원</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>177,820원</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>179,075원</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>배당/가치(안전)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>✂️ 부분 매도 (고점대비 5%하락)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SK텔레콤 (국내 통신/고배당)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>87,400원</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>87,400원</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>108,100원</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>96,845원</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>102,695원</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>배당/가치(안전)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>✂️ 부분 매도 (고점대비 5%하락)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>한미반도체 (사용자 추가)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1주</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>217000</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-27000</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>219,500원</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>-10.95</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>101%</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>219,500원</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>361,000원</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>284,175원</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>284,050원</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t>342,950원</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>성장(공격)</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>✂️ 부분 매도 (고점대비 5%하락)</t>
         </is>
@@ -2305,17 +2549,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 20:51:58 GMT</t>
+          <t>Thu, 02 Jul 2026 07:03:02 GMT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>한국경제TV</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[뉴욕증시] AI 컴퓨팅 용량 남아돈다는데…반도체주 급락</t>
+          <t>성공투자 오후증시</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2325,24 +2569,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE54Y2k3Sjc1RnNjYnJuY2RjdHJRRHAtZVhFWnZKOHV2NVo1VDdUWEJOaFdPTlg0WG9JbFBSM0V6a3pJUTZDcUxWSFFhcDViYkJPU1h2TTZOT2lFdkNJOU4xTDIxd1A3Z1Nlc3loVWpESUI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxObHMxYkx2MmhLT2dwd0w2Qm5ZeVhTREo1bkxNNHlhNk40VXRnS1psSlVDWHlqTHoxeXV1Vi1Vd1lJY1RxN3hhaWotM3BNMlgydnJrbFNNa3NmeEw2TEZYMGUtR3p5YzNHdkxTSEpScmhQM0NReHlsU1RkTkw2MzNEU2YwSkFHanlOclh2eGtkYTdpbW1kbXpNM1pSLV9xR2hyMTdj?oc=5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:55:00 GMT</t>
+          <t>Wed, 01 Jul 2026 20:51:58 GMT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>조선일보</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>"증시 흔들려도 반도체는 믿는다"...파킹형 ETF에서 돈 빼고, 반도체 ETF 산다</t>
+          <t>[뉴욕증시] AI 컴퓨팅 용량 남아돈다는데…반도체주 급락</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2352,24 +2596,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOUHo5elN3Y1FkTVhIYUNlWGhjNWpBZzd5TlBWZmd2TFhFWGlRRjJidUNYZWV2elBtbnlnZVJ5V3ZWal9UU1R5OUhvdzlXNURjaDJwQVJWMUl5TmhTMWJYQU9nMHFjVnBzVzhZaThRTGhxVXdpUjNQb2pFMnFHaGcxQg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE54Y2k3Sjc1RnNjYnJuY2RjdHJRRHAtZVhFWnZKOHV2NVo1VDdUWEJOaFdPTlg0WG9JbFBSM0V6a3pJUTZDcUxWSFFhcDViYkJPU1h2TTZOT2lFdkNJOU4xTDIxd1A3Z1Nlc3loVWpESUI?oc=5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 01:47:58 GMT</t>
+          <t>Thu, 02 Jul 2026 08:32:12 GMT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>"우대금리와 함께 쿠폰도 챙기세요"…iM뱅크, '착착통장' 출시</t>
+          <t>(보도설명) 정부의 '26년 경제전망은 아직 정해진 바 없음을 알려드립니다.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2379,51 +2623,51 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBudm5PQjE0R19pVnBxVHl3OWxGbnF0YnlhMzVJRFBDNm5PNFNzTlQ1aldtczRDTDMzdkFpZWMya3M4OG9SSFlyWi1rTHZwU0c2WkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFBaRXNfb3NnYTlpZlY5aTItZmdhZjVXU3JrWF9BdHhSNEJydnhGVU9Ja2ZTYUllYXZ2SUxWSUZoVE9NUy1BbFprOHpzWU1xeHhZZjRSSkFYZGZhLW00aDZBU05RWUJzX25sMXprcWpaaw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 22:13:11 GMT</t>
+          <t>Thu, 02 Jul 2026 08:08:11 GMT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[증시전략] 메모리 가격 하락?…삼전닉스 팔까 말까, 전망은?</t>
+          <t>오늘의 증시</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBZeklJWEthcGdoNF92TmtyWVJDYVV6QWpNS1YzajM1eVBQVlhYdUZFYjF5RG9JbkN4MkpBT3pBR1pUd3Z4ZVBIamxYbHo2VlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBrUVkxZHN4RmpLbWRPSy1YRmZ2NklIYkJUcjNtVVJQU0xERllCbGJMeUR6MmVnNVJDU1pTNUhqRUxxUkNlelpBR2F6dDhIdVpwcDJSa016d3RTVkRwUkczREtlWUtpSzBNb2dJMWdIVVJJcW5xVkdGbg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:13:35 GMT</t>
+          <t>Thu, 02 Jul 2026 07:20:50 GMT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>한성숙, 첫 비상경제점검회의 주재‥"호르무즈 남은 2척 끝까지 챙길 것"</t>
+          <t>뜨거워진 日증시에…해외 투자자·자국 개미 함께 몰렸다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2433,24 +2677,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE83eVk4a0VLNTI3VzAxcTlycUxMaktwTElrTE51UThSU0lhZk5BeGJwM0lpY1NmNGFwUWJ1MDBnQVEtbjVIYVRYeW16dzljckhiQ2laMTlVUlVGVjh3Z1Q1Z1FVb3I0Q0hRanh5NkhLcGZJQ2lMbWJOZ9IBeEFVX3lxTE1FNDJ4Ymk0MWR3UlVYcC0xTXNCbnVMUUxmeXY3NXVwZVRuMnE3a2tNZ0xsVVZZZVNkRUJqWG1yRG1Xc1dWa1o1U0MxX1JUMWd4ODJ1R01NeTBZd0RiRllVbndPdHNEVXEzQjVYcmo3TlhtT0RRV3RZcg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1wV3BjSVVfWHF5dmNwRFBoWGhfbXBRcGxTZU93VS1EeUZJNkVqVEhLV1ZpVGV0akJab19sZlJQaGJCdzVFbzJ1bUhtVVZUWlV0R2NPZDd2WnNnZzjSAWBBVV95cUxOQ3pFYjNYVjV4bG9zQktrZEFmTmJ3ZzRMQWpIYk5xWnJDZnBKTGpLZzhIV3dzZFZqVEwtNFExWnBJNXNEeDgzWHhhZzQwVXZSclpqTDZXX0RCdkZHNGc5c24?oc=5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:05:41 GMT</t>
+          <t>Thu, 02 Jul 2026 07:30:00 GMT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>한국개발연구원(KDI)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
+          <t>26년 국내 GDP 성장률 3.0%로 상향조정 - 경제 브리프</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2460,24 +2704,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1nR2xubXFiSkZYMk4zOW5aaVpraEJSQ3BqUW1hZGljNXpqRkZaSm40MGNOM2dfYi11Tk9UeXZNNm8wc3ZVVFJPWlJUQm9GaWluNmhJcFNIdXpJSUnSAWBBVV95cUxQZmR6YU41aTdDRmtwYzVoVkVGemQyVWxDaHFUb0pKMWJEeWFGWWFjZHI4MmViN3lQSUQyLWpfRWxsdTZ5T1NXMVJGYTdWaGgwZmh4OVFxLTF5dk1HSVpkckU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE9DUXB0bzU4dDh1cHVaMWNHd2pvQzBWVE56S3lKbHVPU1l2OEJJYUZZMmhqMnpMMWI4NjJFcmVZX3BmX1o1Y3o4bEl3QWMwdTBKeEZHa09iWTR2Vmg0MG9YVGZYVzAwYzNNRS1V?oc=5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 21:55:00 GMT</t>
+          <t>Thu, 02 Jul 2026 06:38:15 GMT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>농민신문</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>(출연) [스타트 경제] 환율, 또 금융위기 후 최고...장중 1,560원까지 위협</t>
+          <t>충북농협, 특별우대금리 제공 ‘NH골든찬스예금’ 출시</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2487,78 +2731,78 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE15ZW9lYkUwVlpRN2lvTUlTUzFvSThLM0VtQkpHQVBvY3lqVDhFNkpnWE03LWtpT05od1NiN0lrRG9LdWJLZzZrcFl5VU00WEJyWS1kb3hmSUJMcF90Mnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBOT3dDdVZuRU4tS2FkaFgtTS1MWFBfV1ZxdEpNNDdHc3BHODBiZV81WGF2ZmRtQ3kyMHBhdlEwTmhyeXMzYkV0X09FenpDWFp5NlM4TGw5c1JtZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:21:23 GMT</t>
+          <t>Thu, 02 Jul 2026 05:02:00 GMT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>지디넷코리아</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>美 반도체 주식 무더기 폭락…"메타발 악재 직격탄"</t>
+          <t>ECB 위원 금리동결 시사…"7월엔 변화 없을 것"</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9qWE54WjVNbDhCTmxtcW5FVllWTFBTSXdNZ2ZNczhNd3BtdjJ5dUNzZmpldHBDdGpHSWJOeDZzY2RhcndYNnZIRFFYZWhWY2tQLV9KX3hR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5DeklTNnJKT3l4THBBY08xYkFrNnZ0NS1FYllxUm1SS1UxVHhxd3h2LXB4eE5mVlBzLWl2bDEwVUh3enlyelpQMjRtVzc4dk81Q2tXSEpQbWw3Rmc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 02:07:08 GMT</t>
+          <t>Thu, 02 Jul 2026 08:14:07 GMT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KB Think</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>日 국채금리 일제히 상승…10년물 표면금리 29년 만에 최고</t>
+          <t>[亞증시-종합] 기술주 조정에 대부분 하락…홍콩만 상승</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>긍정적 (호재)</t>
+          <t>중립</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9IajBWQVpGaFlaLWhTWFJsMk16VERDa0twdmo1em5jNXFNejB0THNXWU5OM0p3cW9EVWN2ZmgxR0NxZWZjMXpUelltcG5hYWxyS2c0Z1YtNXBUVWtiMnJUT2RXMEhwMWxUNTBOcDlmTG1WZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1OZ3hIT0MxVUZTbXd1TVVFRHdQZGZEMk1JR05PTTY5aUNIVENDaUxWb1ZoSGtnT080QmdWQk1ER19Del80aEZSOE1HN0Z5bGhFVmdoTXR1UHZzVVE2azMxcVlwNmV2dC1XalFCVDBOWGE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 01:51:00 GMT</t>
+          <t>Thu, 02 Jul 2026 07:30:00 GMT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>에너지경제신문</t>
+          <t>대한민국 정책브리핑</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>“금리도 증시도 도왔다”...금융지주, 상반기 ‘최대 실적’ 예약</t>
+          <t>우리 경제가 정상화될 때까지 비상한 각오로 정책을 추진하겠습니다 - 카드/한컷 | 멀티미디어</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2568,24 +2812,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5RRTlpdE9kc1JTT1ZZczZoVGN1RGJwbVNVRm9YZThIZ3d6UElEZkNhZWQ0SWIzcUpXZ1pBaERETGNIRHZxR24wWFh3TGEtdTJzR25nZXN1ZVJUenc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNRmFkQ2Qxc1o0Z3VTV0pYalF4b2J5eTUxT3hHNjJENFFzblFXajhwZjdlbGh4ZDZuanJjVU5ZUm1Ud1hORjRaYWxjTlRPNGZFdEJjV1VEUEdzN0JoVVNHTzRlcFJVcTRFcnFsU2JDaXFwb1E5NHUtdUxvb0FmdmFEY3pFcDBGZkxHX2hB?oc=5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:24:11 GMT</t>
+          <t>Thu, 02 Jul 2026 07:30:00 GMT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>한국개발연구원(KDI)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>국민연금 리밸런싱 첫날, 연기금 2천179억원 순매도…얼마나 이어질까</t>
+          <t>최근 대만경제 고성장 특징과 한국에 대한 시사점</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2595,14 +2839,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5kM3RVbWZkQ29wc2dTYzI2YWVrN2VHTUVlaVVkSUxFdURJWk0yOTZiVDB2aW85VktzbXVDUUFfVFg3QmJYaU5lT2lnV0E2d2JwbFRIbEZXczFvR3R1S1lQWUtNTndYOFdXbVhWNVJLSzQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE1rUWpUR2tzVjgwYmJzUzhSZmFrZWJtYS1PUDlDLTF1X3ZjbDdid3RoX2R1dWdaQmgwOFpPLUl5SE1vcGYzLVc5WWFRR1Exb01wQk1vbUhBRHJIZGdUQzVhZnhYamdleW9uQm1z?oc=5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:41:39 GMT</t>
+          <t>Thu, 02 Jul 2026 08:22:24 GMT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2612,7 +2856,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>오늘의 증시</t>
+          <t>8천 깨진 코스피‥"급등에 불안, 시장 과잉반응" [경제쏙]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2622,78 +2866,78 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFA1MWtmcmxtYUU4NGlyQTdmbG5uLWhtbXpwMTNqZU4yOE0zX1g3Z0lKc1I5VnJvYjgzeFZ2WG9sWU9ZNDhtR0xPSlNaWTN1Vk9reEhhbXJGSWhaOFY1Y3ZsSEs2UUxmVlRMNUUwQTdlaDk3OHg3QXp3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE03YzJISE4wZ1FKZG1KNzV5Tkwtd19UY0ZJekg5V1FjdHBmVXk1MGxZT0h2a2pHczBZT29tSDBveXUzWmFBbi1Qc3ZlZmtTYVBlVl9jZ3ZjNnlqNThwUmdFV05FZVJiYTlWZjJZcHlVbTdTOEJGZVdULQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 20:58:01 GMT</t>
+          <t>Thu, 02 Jul 2026 07:57:06 GMT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>v.daum.net</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[뉴욕증시]반도체 업종 울자 일제히 하락 마감…워시 발언에 주목</t>
+          <t>소비자 물가 상승에도 국고채 금리↓…3년물 연 3.747%(종합)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>부정적 (악재)</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTFBBdmYzcUE2TEtFMmpIRlc5X0VndUljeWZUa0Q5MXJWemU2YVk4ekJzM29jclotY1VBb21kdXlUbmczUDZwcWNNYnRiLWYwQW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9nNWlIdXF4NzlUVFdjM3hEQ1VJa0xMQm5UYzZNNFFVRjRfLUNGWS1FYThpVDdGYm0zQXQ4UlkwU0JlaC1NWm8yQm5uN1lMb2lUTHZfUTAzbDB6clU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:06:08 GMT</t>
+          <t>Thu, 02 Jul 2026 07:42:24 GMT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>워시 "생애 최대 경제 격변기…AI 혁명 1∼2회"</t>
+          <t>BofA CEO "연준 세 차례 금리 인상 전망에도 침체 없다"</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE4taGJydHRfVmgwU0puMDI4T243UlE5WjZqcTlLTXp1bkNXNS1NbmN0a2tEQ3otU0xqRFdPMWZhR0pQc1NqcEFzQWN6SWhiUHJuWG53cWQ1TzVTaFnSAWBBVV95cUxOTDNqODVBaHRyUi1SRnQ4SWh2TXJwZ1RtNXRzbzJJbS1iUTRMNDA1ZUJvNlF0aVlpTlFwaTdwNndSZFROSEJIcHZNNm96ZF9WZl8wLTFxLWNLOU53bUMtNzE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1CR2RHQXQ4U2ZNU2MySC1WZkpVNElTOUo2bGNBSVE3UUN2V012eVBneXFvVkNyVlBiRFBiTWJCS0VnaW5XWkFDeFNERnJMZy1seGNacG94bmxOdTM5anJmQ1NFR3BJX0NPU1VfSnBZbk0?oc=5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:44:51 GMT</t>
+          <t>Thu, 02 Jul 2026 08:05:10 GMT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>어린이 경제박사 되세요... 11일 경제교실 개최</t>
+          <t>美개미도 韓주식 '직구'한다…IBKR, 넥스트레이드서 주식거래 개시</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2703,14 +2947,14 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE9XblNZWWkxaUNIcVZDaEpEbldHbWJwa29mSXhtck9ac3NYUm0tR1VKQlhxOWRHRElmcEpjUThWVlpGLUtvNFRKRDA1NXdnaG1RV0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5aQ1BnSGFZUkdaYWlDZGYwcG04LU1jRV9BN2lsSE9Yb184UFB6VEJubUlPMlZHV3AtelhjTkcwdjFQTm5TRzRhVmF3MmF4b0JPZHNDRTQ4OXR5N0ZSenR3MXJUUmdITGItd2ZpeHVmRFo?oc=5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 23:01:58 GMT</t>
+          <t>Thu, 02 Jul 2026 07:21:19 GMT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2720,7 +2964,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[뉴욕마켓워치] '컴퓨팅 용량이 남네?' 반도체 투매…주식·채권↓달러↑</t>
+          <t>유럽증시, 美고용 발표 앞두고 혼조…유로스톡스 0.01%↑</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2730,41 +2974,41 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9EVi1JTE1obG5wc1BsSU9TeDdVQmpnSkdPWE9MWWxVZkYzeTZieThpMFpsMXVpQUVraGlBekNnZ2V5X0tGR09VR0JxOTd1dzVvUEZVTGNZc0xxU3VPRXlJcE1iRkZrZE9tTEkzX2NRT0g?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1XX2RkLTVGY0QxZlVQWkZ5b0lNZ1A0MVEzeHdlZVB5NzlHUlZJUXI0TVdaM19mUjlHeFFrMFQ4bDJ5cXNLQkxJY2tTWjFtUzdnR0tSR19jb1h2Y3FEZklKZzMxNXhmMlcyaUpJOXN2b0fSAXRBVV95cUxOTy1FY2xYSkxmQlQtUE10a1lWUmdwTGVwMnAtYjd5aHluRDJaSnRFRU85YWg3N3lDUWFKaUZQQmJoajlBa3h3akRWNlNfb0ctQVFmV1pJUE5ZNGtMd3pyLXhSTkhKWG1RUER5YWpHRTh5MXNPZA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wed, 01 Jul 2026 21:00:54 GMT</t>
+          <t>Thu, 02 Jul 2026 06:54:50 GMT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>뉴욕증시, 반도체주 매도에 약세 마감…마이크론 10% 급락(종합)</t>
+          <t>[증시_마감] 코스피, 外人·기관 동반 매도에 7.89% 급락…코스닥 6%대 하락</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1VcGFiVW9IV1BGVkpCQlExR2NXcjRQYXVMSHpET18xZ3hKc1ZYTGNPN0s5NTBiUUE0ckdWT3pqZ0Q2UEFyd0k4VjE2dmRWVkNNbFhBdGNlMUF0Q2_SAWBBVV95cUxNNFQ0TE5pUWtBUHo2MEVVQXZmMGQtZGJkX3M2YnZ5SEVXZUY5WFFLUEdtbTRveUI3c1FjVEJQNEw1ZlFyZUZaWlJ4d0pKbWhiVG5wU01pbzY5MUhtcUxoNXQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0yRnhqQnM0cDhCSTNRTHRTTHlNdTNlYUdINEJ6MGVSSnNNblR4c19jSVVkSzlCemxHSnZ4VXBfQXdWc2NLV3RUX1p1UFc4QXVxMG1IVS1pak51dXFtOXZ5NmpxYjM5eEhxcGs4M2loNGc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 03:24:29 GMT</t>
+          <t>Thu, 02 Jul 2026 07:58:47 GMT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2774,24 +3018,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>핌코 "AI, 실질 중립금리 높이는 게 아니라 낮춘다…안전자산 수요↑"</t>
+          <t>"韓 수출 호조에 4% 성장 가시권…연내 3번 금리인상 가능성 높아져"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>긍정적 (호재)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5mbGc1dVh4WVd0NHlEOTlIV3luZFhlcGFBUVBDQ2tWeUozTURjaUNBSjhydUI2RDIyN2hiaFM1QllDM2JoaV9WZWxyTmhyWDFMQjZIbm4wc1BTY2U0VVVMRzEta3NNM1Q1UGt1NUh0b3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1hX2ZJMGhuR0FfTDFyczB4MjRTZ0tEdXFDLUtzcjFLeEk1dnNMWHJ4cVN1NWRYdWkxZXpodTVCSk9Pdkk0T25lYXI5LU5Kc3Y1bllYZWdjUXBMSHQ0RUx3UEtRdmpWTExQeGNmRDloMFjSAXRBVV95cUxOR295UmVROUszdWhzSzFZVmQxUks3bDlULTFlNUlvMUFkSUQ3Q2xhLVlEN3ozVVhSamYySjZPZlVjUVFvbk85RUQ1YjlKa0RHOWZfa0ZUQmNQbm1fdFl0V0t5SXJ1UXk2NElVakVSQXdia2NyOQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Thu, 02 Jul 2026 00:03:22 GMT</t>
+          <t>Thu, 02 Jul 2026 07:06:27 GMT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2801,17 +3045,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[변액보험 상반기] 주식시장 훈풍 지속…라이나생명 수익률 선두</t>
+          <t>[중국증시-마감] 반도체 투매에 2%대 하락</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>중립</t>
+          <t>부정적 (악재)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFAxUmxPSzFMak9XZ2htaVhTeTR4OHpmaTNlMWZVOWdGSjJDdGpxZndXY3A1RHhobW9RSEpzNEN4emE3cktIVDdYNndPMGpRRl9xa2FuS1JOWEU3WGI4LVdtcWYzVk41RzY4aHJtVS10OUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5WU2U4ZHVIQ2tVTFZmWmNsamFsMnBGWnFqdG9UQkFWOXM1QTlsRlF3X1dyc19PRDZEakxTTExYMWFOOWw1SG1kU3FSZWJKOVVtUXNieFNHSGd3M1FvZk5hM1hMQ0hpOWtfbGtBZHhjemU?oc=5</t>
         </is>
       </c>
     </row>
@@ -2881,21 +3125,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AI/반도체 (기술)</t>
+          <t>결제/핀테크 (소비지표)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AI, 🛍️소비/매출폭발, 반도체</t>
+          <t>🛍️소비/매출폭발, 소비, 카드</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SK하이닉스, 한미반도체, 이수페타시스, 삼성전자</t>
+          <t>카카오페이, 네이버페이, KG이니시스, NHN KCP</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -2906,7 +3150,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>환율, 🌱성수기/계절수혜, ✈️유가하락수혜</t>
+          <t>✈️유가하락수혜, 🌱성수기/계절수혜</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2915,27 +3159,27 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>원전/전력기기 (인프라)</t>
+          <t>K-푸드/식품 (수출/소비)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>🌱성수기/계절수혜</t>
+          <t>🛍️소비/매출폭발, 수출</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LS일렉트릭, HD현대일렉트릭, 두산에너빌리티, 효성중공업</t>
+          <t>삼양식품, CJ제일제당, 대상, 빙그레, 농심</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2976,11 +3220,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.18</v>
+        <v>1.12</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KB금융 (+8.01%)</t>
+          <t>KB금융 (+4.1%)</t>
         </is>
       </c>
     </row>
@@ -2991,11 +3235,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.16</v>
+        <v>0.03</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TIGER 미국S&amp;P500 (+0.16%)</t>
+          <t>TIGER 미국S&amp;P500 (+0.03%)</t>
         </is>
       </c>
     </row>
@@ -3006,11 +3250,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.04</v>
+        <v>-0.11</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TIGER 인도니프티50 (-0.04%)</t>
+          <t>TIGER 인도니프티50 (-0.11%)</t>
         </is>
       </c>
     </row>
@@ -3021,11 +3265,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.26</v>
+        <v>-0.14</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KODEX 미국달러선물 (-0.22%)</t>
+          <t>KODEX 미국달러선물 (-0.09%)</t>
         </is>
       </c>
     </row>
@@ -3036,41 +3280,41 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.25</v>
+        <v>-1.8</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LG에너지솔루션 (+2.59%)</t>
+          <t>LG에너지솔루션 (+1.72%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>성장(공격)</t>
+          <t>기후/식량(방어)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.59</v>
+        <v>-3.73</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NAVER (+2.08%)</t>
+          <t>MOO (-0.27%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>기후/식량(방어)</t>
+          <t>성장(공격)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2.7</v>
+        <v>-4.29</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MOO (-0.27%)</t>
+          <t>NAVER (+1.27%)</t>
         </is>
       </c>
     </row>
@@ -3081,11 +3325,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-6.2</v>
+        <v>-9.06</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>삼성전자 (-6.2%)</t>
+          <t>삼성전자 (-9.06%)</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3143,7 +3387,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5,060원</t>
+          <t>4,900원</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3152,7 +3396,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13.2</v>
+        <v>16.9</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -3160,6 +3404,34 @@
         </is>
       </c>
       <c r="F2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TIGER 미국테크TOP10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>33,050원</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>31,070원</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>✅ 보유 및 분할 매수</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>